<commit_message>
Presets, panel safety checks, safer Push Data, docs and tests
</commit_message>
<xml_diff>
--- a/Params/Mouse_Room_Params.xlsx
+++ b/Params/Mouse_Room_Params.xlsx
@@ -446,10 +446,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX14"/>
+  <dimension ref="A1:AY14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="13.57142857142857" customWidth="1" min="1" max="49"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,245 +461,250 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Preset</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Protocol</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Session_Type</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Air_Puff_Contingency_Rule</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>AntiBias</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Distribution</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Stim_Type</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Nb_Of_Stim</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Emulator</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Show_Contingency_Switches</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Sound_Contingency</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Sound_Air_Puff_Contingency</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Working_Memory_Type</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Sound_Duration</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>AntiBias_Exp_Rate</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>AntiBias_Window</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>AntiBias_Sigmoid_Slope</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Agent_Sim</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Agent_Performance</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Agent_Bias</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Stim_Dur_Staircase</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Stim_Dur_Staircase_Perf_Thresh</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Stim_Dur_Staircase_Step</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Min_Stim_Dur</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Timeout_Duration</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Response_Window</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Stim_Range_Min</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Stim_Range_Max</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Go_Cue_Duration</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Visualiser_Window_Size</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Stable_Start</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Stable_Start_Window</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Max_Trials_Consec</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Stable_Stim_Dist_Boundary</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Opto_ON</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>Opto_Type</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Zapit_Nb_Conditions</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>Perc_Opto_Trials</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>Light_Freq (Hz)</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>Opto_Onset_1</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>Opto_Onset_2</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>Opto_Offset_1</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>Opto_Offset_2</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>Opto_Duration</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>Stimulation_Site</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>Stimulation_Type</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>Rig</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>Early_Lick_Abort</t>
         </is>
@@ -712,42 +718,42 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Habituation</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>2</v>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -755,97 +761,102 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>300</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>1</v>
       </c>
-      <c r="Q2" t="n">
-        <v>30</v>
-      </c>
       <c r="R2" t="n">
+        <v>30</v>
+      </c>
+      <c r="S2" t="n">
         <v>1.75</v>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T2" t="n">
-        <v>0.8</v>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V2" t="n">
         <v>0.5</v>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W2" t="n">
-        <v>0.8</v>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X2" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y2" t="n">
         <v>50</v>
       </c>
       <c r="Z2" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA2" t="n">
         <v>10</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AB2" t="n">
         <v>3</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>10</v>
       </c>
-      <c r="AC2" t="n">
-        <v>50</v>
-      </c>
       <c r="AD2" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE2" t="n">
         <v>82</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AF2" t="n">
         <v>300</v>
       </c>
-      <c r="AF2" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AG2" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH2" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH2" t="n">
+      <c r="AI2" t="n">
         <v>20</v>
       </c>
-      <c r="AI2" t="n">
+      <c r="AJ2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ2" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr">
+      <c r="AK2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -859,42 +870,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Lick_To_Release</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>2</v>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -902,97 +913,102 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>300</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>1</v>
       </c>
-      <c r="Q3" t="n">
-        <v>30</v>
-      </c>
       <c r="R3" t="n">
+        <v>30</v>
+      </c>
+      <c r="S3" t="n">
         <v>1.75</v>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T3" t="n">
-        <v>0.8</v>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V3" t="n">
         <v>0.5</v>
       </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W3" t="n">
-        <v>0.8</v>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X3" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y3" t="n">
         <v>50</v>
       </c>
       <c r="Z3" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA3" t="n">
         <v>2</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
         <v>3</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>10</v>
       </c>
-      <c r="AC3" t="n">
-        <v>50</v>
-      </c>
       <c r="AD3" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE3" t="n">
         <v>82</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AF3" t="n">
         <v>300</v>
       </c>
-      <c r="AF3" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AG3" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH3" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH3" t="n">
+      <c r="AI3" t="n">
         <v>20</v>
       </c>
-      <c r="AI3" t="n">
+      <c r="AJ3" t="n">
         <v>3</v>
       </c>
-      <c r="AJ3" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr">
+      <c r="AK3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1006,42 +1022,42 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Three_And_Three</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>2</v>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K4" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -1049,97 +1065,102 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>300</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>1</v>
       </c>
-      <c r="Q4" t="n">
-        <v>30</v>
-      </c>
       <c r="R4" t="n">
+        <v>30</v>
+      </c>
+      <c r="S4" t="n">
         <v>1.75</v>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T4" t="n">
-        <v>0.8</v>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V4" t="n">
         <v>0.5</v>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W4" t="n">
-        <v>0.8</v>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X4" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y4" t="n">
         <v>50</v>
       </c>
       <c r="Z4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA4" t="n">
         <v>2</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AB4" t="n">
         <v>3</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AC4" t="n">
         <v>10</v>
       </c>
-      <c r="AC4" t="n">
-        <v>50</v>
-      </c>
       <c r="AD4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE4" t="n">
         <v>82</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AF4" t="n">
         <v>300</v>
       </c>
-      <c r="AF4" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AG4" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH4" t="n">
+      <c r="AI4" t="n">
         <v>20</v>
       </c>
-      <c r="AI4" t="n">
+      <c r="AJ4" t="n">
         <v>3</v>
       </c>
-      <c r="AJ4" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK4" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr">
+      <c r="AK4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1153,44 +1174,44 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Full_Task_Cont</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>8.0</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -1198,133 +1219,138 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>300</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>1</v>
       </c>
-      <c r="Q5" t="n">
-        <v>30</v>
-      </c>
       <c r="R5" t="n">
+        <v>30</v>
+      </c>
+      <c r="S5" t="n">
         <v>1</v>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T5" t="n">
-        <v>0.8</v>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V5" t="n">
         <v>0.5</v>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W5" t="n">
-        <v>0.8</v>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X5" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y5" t="n">
         <v>50</v>
       </c>
       <c r="Z5" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA5" t="n">
         <v>2</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AB5" t="n">
         <v>3</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AC5" t="n">
         <v>10</v>
       </c>
-      <c r="AC5" t="n">
-        <v>50</v>
-      </c>
       <c r="AD5" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE5" t="n">
         <v>82</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AF5" t="n">
         <v>300</v>
       </c>
-      <c r="AF5" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG5" t="inlineStr">
+      <c r="AG5" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH5" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH5" t="n">
+      <c r="AI5" t="n">
         <v>20</v>
       </c>
-      <c r="AI5" t="n">
+      <c r="AJ5" t="n">
         <v>2</v>
       </c>
-      <c r="AJ5" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+      <c r="AK5" t="n">
+        <v>0.8</v>
       </c>
       <c r="AL5" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
           <t>Zapit</t>
         </is>
       </c>
-      <c r="AM5" t="n">
+      <c r="AN5" t="n">
         <v>1</v>
       </c>
-      <c r="AN5" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP5" t="inlineStr">
+      <c r="AO5" t="n">
+        <v>30</v>
+      </c>
+      <c r="AQ5" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="AR5" t="inlineStr">
+      <c r="AS5" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="AS5" t="inlineStr">
+      <c r="AT5" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AU5" t="inlineStr">
+      <c r="AV5" t="inlineStr">
         <is>
           <t>ALM</t>
         </is>
       </c>
-      <c r="AV5" t="inlineStr">
+      <c r="AW5" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="AX5" t="inlineStr">
+      <c r="AY5" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1338,42 +1364,42 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Full_Task_Cont</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>8</v>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -1381,133 +1407,138 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>150</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>1</v>
       </c>
-      <c r="Q6" t="n">
-        <v>30</v>
-      </c>
       <c r="R6" t="n">
+        <v>30</v>
+      </c>
+      <c r="S6" t="n">
         <v>0</v>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T6" t="n">
-        <v>0.8</v>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V6" t="n">
         <v>0.5</v>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W6" t="n">
-        <v>0.8</v>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X6" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y6" t="n">
         <v>50</v>
       </c>
       <c r="Z6" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA6" t="n">
         <v>2</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AB6" t="n">
         <v>3</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AC6" t="n">
         <v>10</v>
       </c>
-      <c r="AC6" t="n">
-        <v>50</v>
-      </c>
       <c r="AD6" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE6" t="n">
         <v>82</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AF6" t="n">
         <v>300</v>
       </c>
-      <c r="AF6" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG6" t="inlineStr">
+      <c r="AG6" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH6" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH6" t="n">
+      <c r="AI6" t="n">
         <v>20</v>
       </c>
-      <c r="AI6" t="n">
+      <c r="AJ6" t="n">
         <v>3</v>
       </c>
-      <c r="AJ6" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK6" t="inlineStr">
+      <c r="AK6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL6" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AL6" t="inlineStr">
+      <c r="AM6" t="inlineStr">
         <is>
           <t>Zapit</t>
         </is>
       </c>
-      <c r="AM6" t="n">
+      <c r="AN6" t="n">
         <v>1</v>
       </c>
-      <c r="AN6" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP6" t="inlineStr">
+      <c r="AO6" t="n">
+        <v>30</v>
+      </c>
+      <c r="AQ6" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="AR6" t="inlineStr">
+      <c r="AS6" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="AS6" t="inlineStr">
+      <c r="AT6" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AU6" t="inlineStr">
+      <c r="AV6" t="inlineStr">
         <is>
           <t>ALM</t>
         </is>
       </c>
-      <c r="AV6" t="inlineStr">
+      <c r="AW6" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="AX6" t="inlineStr">
+      <c r="AY6" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1521,42 +1552,42 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Full_Task_Cont</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>8</v>
       </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -1564,133 +1595,138 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>150</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>1</v>
       </c>
-      <c r="Q7" t="n">
-        <v>30</v>
-      </c>
       <c r="R7" t="n">
+        <v>30</v>
+      </c>
+      <c r="S7" t="n">
         <v>0</v>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T7" t="n">
-        <v>0.8</v>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V7" t="n">
         <v>0.5</v>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W7" t="n">
-        <v>0.8</v>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X7" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y7" t="n">
         <v>50</v>
       </c>
       <c r="Z7" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA7" t="n">
         <v>2</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AB7" t="n">
         <v>3</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AC7" t="n">
         <v>10</v>
       </c>
-      <c r="AC7" t="n">
-        <v>50</v>
-      </c>
       <c r="AD7" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE7" t="n">
         <v>82</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AF7" t="n">
         <v>300</v>
       </c>
-      <c r="AF7" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG7" t="inlineStr">
+      <c r="AG7" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH7" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH7" t="n">
+      <c r="AI7" t="n">
         <v>20</v>
       </c>
-      <c r="AI7" t="n">
+      <c r="AJ7" t="n">
         <v>3</v>
       </c>
-      <c r="AJ7" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK7" t="inlineStr">
+      <c r="AK7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL7" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AL7" t="inlineStr">
+      <c r="AM7" t="inlineStr">
         <is>
           <t>Zapit</t>
         </is>
       </c>
-      <c r="AM7" t="n">
+      <c r="AN7" t="n">
         <v>1</v>
       </c>
-      <c r="AN7" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP7" t="inlineStr">
+      <c r="AO7" t="n">
+        <v>30</v>
+      </c>
+      <c r="AQ7" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="AR7" t="inlineStr">
+      <c r="AS7" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="AS7" t="inlineStr">
+      <c r="AT7" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AU7" t="inlineStr">
+      <c r="AV7" t="inlineStr">
         <is>
           <t>ALM</t>
         </is>
       </c>
-      <c r="AV7" t="inlineStr">
+      <c r="AW7" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="AX7" t="inlineStr">
+      <c r="AY7" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1704,42 +1740,42 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Full_Task_Cont</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>8</v>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -1747,133 +1783,138 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>150</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>1</v>
       </c>
-      <c r="Q8" t="n">
-        <v>30</v>
-      </c>
       <c r="R8" t="n">
+        <v>30</v>
+      </c>
+      <c r="S8" t="n">
         <v>0</v>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T8" t="n">
-        <v>0.8</v>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V8" t="n">
         <v>0.5</v>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W8" t="n">
-        <v>0.8</v>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X8" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y8" t="n">
         <v>50</v>
       </c>
       <c r="Z8" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA8" t="n">
         <v>2</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AB8" t="n">
         <v>3</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AC8" t="n">
         <v>10</v>
       </c>
-      <c r="AC8" t="n">
-        <v>50</v>
-      </c>
       <c r="AD8" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE8" t="n">
         <v>82</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AF8" t="n">
         <v>300</v>
       </c>
-      <c r="AF8" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG8" t="inlineStr">
+      <c r="AG8" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH8" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH8" t="n">
+      <c r="AI8" t="n">
         <v>20</v>
       </c>
-      <c r="AI8" t="n">
+      <c r="AJ8" t="n">
         <v>3</v>
       </c>
-      <c r="AJ8" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK8" t="inlineStr">
+      <c r="AK8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL8" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AL8" t="inlineStr">
+      <c r="AM8" t="inlineStr">
         <is>
           <t>Zapit</t>
         </is>
       </c>
-      <c r="AM8" t="n">
+      <c r="AN8" t="n">
         <v>1</v>
       </c>
-      <c r="AN8" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP8" t="inlineStr">
+      <c r="AO8" t="n">
+        <v>30</v>
+      </c>
+      <c r="AQ8" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="AR8" t="inlineStr">
+      <c r="AS8" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="AS8" t="inlineStr">
+      <c r="AT8" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AU8" t="inlineStr">
+      <c r="AV8" t="inlineStr">
         <is>
           <t>ALM</t>
         </is>
       </c>
-      <c r="AV8" t="inlineStr">
+      <c r="AW8" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="AX8" t="inlineStr">
+      <c r="AY8" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1887,42 +1928,42 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Full_Task_Cont</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>8</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -1930,133 +1971,138 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>150</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>1</v>
       </c>
-      <c r="Q9" t="n">
-        <v>30</v>
-      </c>
       <c r="R9" t="n">
+        <v>30</v>
+      </c>
+      <c r="S9" t="n">
         <v>0</v>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T9" t="n">
-        <v>0.8</v>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V9" t="n">
         <v>0.5</v>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W9" t="n">
-        <v>0.8</v>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X9" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y9" t="n">
         <v>50</v>
       </c>
       <c r="Z9" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA9" t="n">
         <v>2</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AB9" t="n">
         <v>3</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AC9" t="n">
         <v>10</v>
       </c>
-      <c r="AC9" t="n">
-        <v>50</v>
-      </c>
       <c r="AD9" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE9" t="n">
         <v>82</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AF9" t="n">
         <v>300</v>
       </c>
-      <c r="AF9" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG9" t="inlineStr">
+      <c r="AG9" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH9" t="n">
+      <c r="AI9" t="n">
         <v>20</v>
       </c>
-      <c r="AI9" t="n">
+      <c r="AJ9" t="n">
         <v>3</v>
       </c>
-      <c r="AJ9" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK9" t="inlineStr">
+      <c r="AK9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL9" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AL9" t="inlineStr">
+      <c r="AM9" t="inlineStr">
         <is>
           <t>Zapit</t>
         </is>
       </c>
-      <c r="AM9" t="n">
+      <c r="AN9" t="n">
         <v>1</v>
       </c>
-      <c r="AN9" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP9" t="inlineStr">
+      <c r="AO9" t="n">
+        <v>30</v>
+      </c>
+      <c r="AQ9" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="AR9" t="inlineStr">
+      <c r="AS9" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="AS9" t="inlineStr">
+      <c r="AT9" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AU9" t="inlineStr">
+      <c r="AV9" t="inlineStr">
         <is>
           <t>ALM</t>
         </is>
       </c>
-      <c r="AV9" t="inlineStr">
+      <c r="AW9" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="AX9" t="inlineStr">
+      <c r="AY9" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2070,42 +2116,42 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Full_Task_Cont</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>8</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K10" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -2113,133 +2159,138 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>150</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>1</v>
       </c>
-      <c r="Q10" t="n">
-        <v>30</v>
-      </c>
       <c r="R10" t="n">
+        <v>30</v>
+      </c>
+      <c r="S10" t="n">
         <v>0</v>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T10" t="n">
-        <v>0.8</v>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V10" t="n">
         <v>0.5</v>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W10" t="n">
-        <v>0.8</v>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X10" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y10" t="n">
         <v>50</v>
       </c>
       <c r="Z10" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA10" t="n">
         <v>2</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AB10" t="n">
         <v>3</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AC10" t="n">
         <v>10</v>
       </c>
-      <c r="AC10" t="n">
-        <v>50</v>
-      </c>
       <c r="AD10" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE10" t="n">
         <v>82</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AF10" t="n">
         <v>300</v>
       </c>
-      <c r="AF10" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG10" t="inlineStr">
+      <c r="AG10" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH10" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH10" t="n">
+      <c r="AI10" t="n">
         <v>20</v>
       </c>
-      <c r="AI10" t="n">
+      <c r="AJ10" t="n">
         <v>3</v>
       </c>
-      <c r="AJ10" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK10" t="inlineStr">
+      <c r="AK10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL10" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AL10" t="inlineStr">
+      <c r="AM10" t="inlineStr">
         <is>
           <t>Zapit</t>
         </is>
       </c>
-      <c r="AM10" t="n">
+      <c r="AN10" t="n">
         <v>1</v>
       </c>
-      <c r="AN10" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP10" t="inlineStr">
+      <c r="AO10" t="n">
+        <v>30</v>
+      </c>
+      <c r="AQ10" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="AR10" t="inlineStr">
+      <c r="AS10" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="AS10" t="inlineStr">
+      <c r="AT10" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AU10" t="inlineStr">
+      <c r="AV10" t="inlineStr">
         <is>
           <t>ALM</t>
         </is>
       </c>
-      <c r="AV10" t="inlineStr">
+      <c r="AW10" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="AX10" t="inlineStr">
+      <c r="AY10" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2253,42 +2304,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Full_Task_Cont</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>8</v>
       </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -2296,133 +2347,138 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>150</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>1</v>
       </c>
-      <c r="Q11" t="n">
-        <v>30</v>
-      </c>
       <c r="R11" t="n">
+        <v>30</v>
+      </c>
+      <c r="S11" t="n">
         <v>0</v>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T11" t="n">
-        <v>0.8</v>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V11" t="n">
         <v>0.5</v>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W11" t="n">
-        <v>0.8</v>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X11" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y11" t="n">
         <v>50</v>
       </c>
       <c r="Z11" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA11" t="n">
         <v>2</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AB11" t="n">
         <v>3</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AC11" t="n">
         <v>10</v>
       </c>
-      <c r="AC11" t="n">
-        <v>50</v>
-      </c>
       <c r="AD11" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE11" t="n">
         <v>82</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AF11" t="n">
         <v>300</v>
       </c>
-      <c r="AF11" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG11" t="inlineStr">
+      <c r="AG11" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH11" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH11" t="n">
+      <c r="AI11" t="n">
         <v>20</v>
       </c>
-      <c r="AI11" t="n">
+      <c r="AJ11" t="n">
         <v>3</v>
       </c>
-      <c r="AJ11" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK11" t="inlineStr">
+      <c r="AK11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL11" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AL11" t="inlineStr">
+      <c r="AM11" t="inlineStr">
         <is>
           <t>Zapit</t>
         </is>
       </c>
-      <c r="AM11" t="n">
+      <c r="AN11" t="n">
         <v>1</v>
       </c>
-      <c r="AN11" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP11" t="inlineStr">
+      <c r="AO11" t="n">
+        <v>30</v>
+      </c>
+      <c r="AQ11" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="AR11" t="inlineStr">
+      <c r="AS11" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="AS11" t="inlineStr">
+      <c r="AT11" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AU11" t="inlineStr">
+      <c r="AV11" t="inlineStr">
         <is>
           <t>ALM</t>
         </is>
       </c>
-      <c r="AV11" t="inlineStr">
+      <c r="AW11" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="AX11" t="inlineStr">
+      <c r="AY11" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2436,42 +2492,42 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Full_Task_Cont</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>8</v>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -2479,133 +2535,138 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>150</v>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>1</v>
       </c>
-      <c r="Q12" t="n">
-        <v>30</v>
-      </c>
       <c r="R12" t="n">
+        <v>30</v>
+      </c>
+      <c r="S12" t="n">
         <v>0</v>
       </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T12" t="n">
-        <v>0.8</v>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V12" t="n">
         <v>0.5</v>
       </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W12" t="n">
-        <v>0.8</v>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X12" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y12" t="n">
         <v>50</v>
       </c>
       <c r="Z12" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA12" t="n">
         <v>2</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AB12" t="n">
         <v>3</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AC12" t="n">
         <v>10</v>
       </c>
-      <c r="AC12" t="n">
-        <v>50</v>
-      </c>
       <c r="AD12" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE12" t="n">
         <v>82</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AF12" t="n">
         <v>300</v>
       </c>
-      <c r="AF12" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG12" t="inlineStr">
+      <c r="AG12" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH12" t="n">
+      <c r="AI12" t="n">
         <v>20</v>
       </c>
-      <c r="AI12" t="n">
+      <c r="AJ12" t="n">
         <v>3</v>
       </c>
-      <c r="AJ12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK12" t="inlineStr">
+      <c r="AK12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AL12" t="inlineStr">
+      <c r="AM12" t="inlineStr">
         <is>
           <t>Zapit</t>
         </is>
       </c>
-      <c r="AM12" t="n">
+      <c r="AN12" t="n">
         <v>1</v>
       </c>
-      <c r="AN12" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP12" t="inlineStr">
+      <c r="AO12" t="n">
+        <v>30</v>
+      </c>
+      <c r="AQ12" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="AR12" t="inlineStr">
+      <c r="AS12" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="AS12" t="inlineStr">
+      <c r="AT12" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AU12" t="inlineStr">
+      <c r="AV12" t="inlineStr">
         <is>
           <t>ALM</t>
         </is>
       </c>
-      <c r="AV12" t="inlineStr">
+      <c r="AW12" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="AX12" t="inlineStr">
+      <c r="AY12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2619,42 +2680,42 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Full_Task_Cont</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>8</v>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -2662,133 +2723,138 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>150</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>1</v>
       </c>
-      <c r="Q13" t="n">
-        <v>30</v>
-      </c>
       <c r="R13" t="n">
+        <v>30</v>
+      </c>
+      <c r="S13" t="n">
         <v>0</v>
       </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T13" t="n">
-        <v>0.8</v>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V13" t="n">
         <v>0.5</v>
       </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W13" t="n">
-        <v>0.8</v>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X13" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y13" t="n">
         <v>50</v>
       </c>
       <c r="Z13" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA13" t="n">
         <v>2</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AB13" t="n">
         <v>3</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AC13" t="n">
         <v>10</v>
       </c>
-      <c r="AC13" t="n">
-        <v>50</v>
-      </c>
       <c r="AD13" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE13" t="n">
         <v>82</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AF13" t="n">
         <v>300</v>
       </c>
-      <c r="AF13" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG13" t="inlineStr">
+      <c r="AG13" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH13" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH13" t="n">
+      <c r="AI13" t="n">
         <v>20</v>
       </c>
-      <c r="AI13" t="n">
+      <c r="AJ13" t="n">
         <v>3</v>
       </c>
-      <c r="AJ13" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK13" t="inlineStr">
+      <c r="AK13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL13" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AL13" t="inlineStr">
+      <c r="AM13" t="inlineStr">
         <is>
           <t>Zapit</t>
         </is>
       </c>
-      <c r="AM13" t="n">
+      <c r="AN13" t="n">
         <v>1</v>
       </c>
-      <c r="AN13" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP13" t="inlineStr">
+      <c r="AO13" t="n">
+        <v>30</v>
+      </c>
+      <c r="AQ13" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="AR13" t="inlineStr">
+      <c r="AS13" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="AS13" t="inlineStr">
+      <c r="AT13" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AU13" t="inlineStr">
+      <c r="AV13" t="inlineStr">
         <is>
           <t>ALM</t>
         </is>
       </c>
-      <c r="AV13" t="inlineStr">
+      <c r="AW13" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="AX13" t="inlineStr">
+      <c r="AY13" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2802,42 +2868,42 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>SOUND_CAT</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Full_Task_Cont</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>alm_control_uni</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="G14" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>Uniform</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>WN</t>
         </is>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>8</v>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -2845,133 +2911,138 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
           <t>Low_Left_High_Right</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Low_Pro_High_Anti</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="O14" t="n">
+      <c r="P14" t="n">
         <v>150</v>
       </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
         <v>1</v>
       </c>
-      <c r="Q14" t="n">
-        <v>30</v>
-      </c>
       <c r="R14" t="n">
+        <v>30</v>
+      </c>
+      <c r="S14" t="n">
         <v>0</v>
       </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="T14" t="n">
-        <v>0.8</v>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="U14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V14" t="n">
         <v>0.5</v>
       </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="W14" t="n">
-        <v>0.8</v>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
       <c r="X14" t="n">
-        <v>50</v>
+        <v>0.8</v>
       </c>
       <c r="Y14" t="n">
         <v>50</v>
       </c>
       <c r="Z14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA14" t="n">
         <v>2</v>
       </c>
-      <c r="AA14" t="n">
+      <c r="AB14" t="n">
         <v>3</v>
       </c>
-      <c r="AB14" t="n">
+      <c r="AC14" t="n">
         <v>10</v>
       </c>
-      <c r="AC14" t="n">
-        <v>50</v>
-      </c>
       <c r="AD14" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE14" t="n">
         <v>82</v>
       </c>
-      <c r="AE14" t="n">
+      <c r="AF14" t="n">
         <v>300</v>
       </c>
-      <c r="AF14" t="n">
-        <v>30</v>
-      </c>
-      <c r="AG14" t="inlineStr">
+      <c r="AG14" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AH14" t="n">
+      <c r="AI14" t="n">
         <v>20</v>
       </c>
-      <c r="AI14" t="n">
+      <c r="AJ14" t="n">
         <v>3</v>
       </c>
-      <c r="AJ14" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AK14" t="inlineStr">
+      <c r="AK14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AL14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="AL14" t="inlineStr">
+      <c r="AM14" t="inlineStr">
         <is>
           <t>Zapit</t>
         </is>
       </c>
-      <c r="AM14" t="n">
+      <c r="AN14" t="n">
         <v>1</v>
       </c>
-      <c r="AN14" t="n">
-        <v>30</v>
-      </c>
-      <c r="AP14" t="inlineStr">
+      <c r="AO14" t="n">
+        <v>30</v>
+      </c>
+      <c r="AQ14" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="AR14" t="inlineStr">
+      <c r="AS14" t="inlineStr">
         <is>
           <t>Feedback</t>
         </is>
       </c>
-      <c r="AS14" t="inlineStr">
+      <c r="AT14" t="inlineStr">
         <is>
           <t>Inter_Trial_Interval</t>
         </is>
       </c>
-      <c r="AU14" t="inlineStr">
+      <c r="AV14" t="inlineStr">
         <is>
           <t>ALM</t>
         </is>
       </c>
-      <c r="AV14" t="inlineStr">
+      <c r="AW14" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="AX14" t="inlineStr">
+      <c r="AY14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>

</xml_diff>

<commit_message>
21 presets from the example sheet, TRAINING.md, tidied example
</commit_message>
<xml_diff>
--- a/Params/Mouse_Room_Params.xlsx
+++ b/Params/Mouse_Room_Params.xlsx
@@ -733,7 +733,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>alm_control_uni</t>
+          <t>control-alm-uni</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">

</xml_diff>